<commit_message>
Update report examples with new JSON data structure and enhance passing report statistics. Modify empty and passing HTML files to reflect updated metrics and diagnostics, and include changes in the passing.xlsx file.
</commit_message>
<xml_diff>
--- a/public/report-examples/passing.xlsx
+++ b/public/report-examples/passing.xlsx
@@ -34,10 +34,19 @@
     <t>transcript_names</t>
   </si>
   <si>
+    <t>n_trans</t>
+  </si>
+  <si>
     <t>target_region</t>
   </si>
   <si>
-    <t>n_trans</t>
+    <t>target_fold_score</t>
+  </si>
+  <si>
+    <t>target_mapped_genes</t>
+  </si>
+  <si>
+    <t>amp_probe</t>
   </si>
   <si>
     <t>amp_probe.part1</t>
@@ -49,7 +58,13 @@
     <t>amp_probe.part3</t>
   </si>
   <si>
-    <t>amp_probe</t>
+    <t>amp_probe_fold_score</t>
+  </si>
+  <si>
+    <t>amp_probe_self_match</t>
+  </si>
+  <si>
+    <t>mRNA</t>
   </si>
   <si>
     <t>mRNA.part1</t>
@@ -61,7 +76,16 @@
     <t>mRNA.part3</t>
   </si>
   <si>
-    <t>mRNA</t>
+    <t>mRNA_part1_tm</t>
+  </si>
+  <si>
+    <t>mRNA_part2_tm</t>
+  </si>
+  <si>
+    <t>mRNA_part3_tm</t>
+  </si>
+  <si>
+    <t>pad_probe</t>
   </si>
   <si>
     <t>pad_probe.part1</t>
@@ -79,36 +103,12 @@
     <t>pad_probe.part3</t>
   </si>
   <si>
-    <t>pad_probe</t>
-  </si>
-  <si>
-    <t>amp_probe_fold_score</t>
-  </si>
-  <si>
-    <t>amp_probe_self_match</t>
-  </si>
-  <si>
-    <t>mRNA_part1_tm</t>
-  </si>
-  <si>
-    <t>mRNA_part2_tm</t>
-  </si>
-  <si>
-    <t>mRNA_part3_tm</t>
-  </si>
-  <si>
     <t>pad_probe_fold_score</t>
   </si>
   <si>
     <t>pad_probe_self_match</t>
   </si>
   <si>
-    <t>target_fold_score</t>
-  </si>
-  <si>
-    <t>target_mapped_genes</t>
-  </si>
-  <si>
     <t>MiPTestGene_907</t>
   </si>
   <si>
@@ -127,6 +127,9 @@
     <t>AAGGGGAGAGAAAGAAAGAGGGAGAGAGAGGAGGGAGAAA</t>
   </si>
   <si>
+    <t>TTTCTCCCTCCTCAAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>TTTCTCCCTCCTC</t>
   </si>
   <si>
@@ -136,7 +139,7 @@
     <t>AGGAAGAGAG</t>
   </si>
   <si>
-    <t>TTTCTCCCTCCTCAAGGAAGAGAG</t>
+    <t>AAGGGGAGAGAAAGAAAGAGGGAGAGGAGGAGGGAGAAA</t>
   </si>
   <si>
     <t>AAGGGGAGAGAAA</t>
@@ -148,7 +151,7 @@
     <t>GAGGAGGGAGAAA</t>
   </si>
   <si>
-    <t>AAGGGGAGAGAAAGAAAGAGGGAGAGGAGGAGGGAGAAA</t>
+    <t>TTTCTCTCCCCTTCCTCTTCCTTCTATCCTCTCTTCCTCTCTCCCTCTTTC</t>
   </si>
   <si>
     <t>TTTCTCTCCCCTT</t>
@@ -166,9 +169,6 @@
     <t>CTCTCCCTCTTTC</t>
   </si>
   <si>
-    <t>TTTCTCTCCCCTTCCTCTTCCTTCTATCCTCTCTTCCTCTCTCCCTCTTTC</t>
-  </si>
-  <si>
     <t>MiPTestGene_947</t>
   </si>
   <si>
@@ -178,10 +178,13 @@
     <t>AAAGGGAAAGGGAGGGGAGGGGAAAAAAGGGGGGAAAGAA</t>
   </si>
   <si>
+    <t>TTCTTTCCCCCCTAAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>TTCTTTCCCCCCT</t>
   </si>
   <si>
-    <t>TTCTTTCCCCCCTAAGGAAGAGAG</t>
+    <t>AAAGGGAAAGGGAGGGGAGGGGAAAAAGGGGGGAAAGAA</t>
   </si>
   <si>
     <t>AAAGGGAAAGGGA</t>
@@ -193,7 +196,7 @@
     <t>AGGGGGGAAAGAA</t>
   </si>
   <si>
-    <t>AAAGGGAAAGGGAGGGGAGGGGAAAAAGGGGGGAAAGAA</t>
+    <t>TCCCTTTCCCTTTCCTCTTCCTTCTATCCTCTCTTCCTTTTTCCCCTCCCC</t>
   </si>
   <si>
     <t>TCCCTTTCCCTTT</t>
@@ -202,9 +205,6 @@
     <t>TTTTCCCCTCCCC</t>
   </si>
   <si>
-    <t>TCCCTTTCCCTTTCCTCTTCCTTCTATCCTCTCTTCCTTTTTCCCCTCCCC</t>
-  </si>
-  <si>
     <t>MiPTestGene_137</t>
   </si>
   <si>
@@ -217,13 +217,16 @@
     <t>AGAGGAAAAGGGAGGAGAGGAGGAAGGGGGAGGGGGAAAA</t>
   </si>
   <si>
+    <t>TTTTCCCCCTCCCGAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>TTTTCCCCCTCCC</t>
   </si>
   <si>
     <t>G</t>
   </si>
   <si>
-    <t>TTTTCCCCCTCCCGAGGAAGAGAG</t>
+    <t>AGAGGAAAAGGGAGGAGAGGAGGAAGGGGAGGGGGAAAA</t>
   </si>
   <si>
     <t>AGAGGAAAAGGGA</t>
@@ -235,7 +238,7 @@
     <t>GGGAGGGGGAAAA</t>
   </si>
   <si>
-    <t>AGAGGAAAAGGGAGGAGAGGAGGAAGGGGAGGGGGAAAA</t>
+    <t>TCCCTTTTCCTCTCCTCTTCCTTCTATCCTCTCTTCCTCTTCCTCCTCTCC</t>
   </si>
   <si>
     <t>TCCCTTTTCCTCT</t>
@@ -244,9 +247,6 @@
     <t>CTTCCTCCTCTCC</t>
   </si>
   <si>
-    <t>TCCCTTTTCCTCTCCTCTTCCTTCTATCCTCTCTTCCTCTTCCTCCTCTCC</t>
-  </si>
-  <si>
     <t>MiPTestGene_188</t>
   </si>
   <si>
@@ -256,10 +256,13 @@
     <t>AGAGAAGAAAGGAGAAGGGAGAGAAGAAGGGAGAAAGGGG</t>
   </si>
   <si>
+    <t>CCCCTTTCTCCCTAAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>CCCCTTTCTCCCT</t>
   </si>
   <si>
-    <t>CCCCTTTCTCCCTAAGGAAGAGAG</t>
+    <t>AGAGAAGAAAGGAGAAGGGAGAGAAGAGGGAGAAAGGGG</t>
   </si>
   <si>
     <t>AGAGAAGAAAGGA</t>
@@ -271,7 +274,7 @@
     <t>AGGGAGAAAGGGG</t>
   </si>
   <si>
-    <t>AGAGAAGAAAGGAGAAGGGAGAGAAGAGGGAGAAAGGGG</t>
+    <t>TCCTTTCTTCTCTCCTCTTCCTTCTATCCTCTCTTCCTCTTCTCTCCCTTC</t>
   </si>
   <si>
     <t>TCCTTTCTTCTCT</t>
@@ -280,9 +283,6 @@
     <t>CTTCTCTCCCTTC</t>
   </si>
   <si>
-    <t>TCCTTTCTTCTCTCCTCTTCCTTCTATCCTCTCTTCCTCTTCTCTCCCTTC</t>
-  </si>
-  <si>
     <t>MiPTestGene_254</t>
   </si>
   <si>
@@ -292,10 +292,13 @@
     <t>AAAGAAGAGGAGAAGAAGGAAGGGGGGAGGAAAAAGGGGA</t>
   </si>
   <si>
+    <t>TCCCCTTTTTCCTGAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>TCCCCTTTTTCCT</t>
   </si>
   <si>
-    <t>TCCCCTTTTTCCTGAGGAAGAGAG</t>
+    <t>AAAGAAGAGGAGAAGAAGGAAGGGGGAGGAAAAAGGGGA</t>
   </si>
   <si>
     <t>AAAGAAGAGGAGA</t>
@@ -307,7 +310,7 @@
     <t>AGGAAAAAGGGGA</t>
   </si>
   <si>
-    <t>AAAGAAGAGGAGAAGAAGGAAGGGGGAGGAAAAAGGGGA</t>
+    <t>TCTCCTCTTCTTTCCTCTTCCTTCTATCCTCTCTTCCTCCCCCTTCCTTCT</t>
   </si>
   <si>
     <t>TCTCCTCTTCTTT</t>
@@ -316,9 +319,6 @@
     <t>CCCCCTTCCTTCT</t>
   </si>
   <si>
-    <t>TCTCCTCTTCTTTCCTCTTCCTTCTATCCTCTCTTCCTCCCCCTTCCTTCT</t>
-  </si>
-  <si>
     <t>MiPTestGene_1172</t>
   </si>
   <si>
@@ -328,10 +328,13 @@
     <t>GAAGGAGGAAGGAGAAGGAAAAGGAAAAGGAGGGGAAAAA</t>
   </si>
   <si>
+    <t>TTTTTCCCCTCCTAAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>TTTTTCCCCTCCT</t>
   </si>
   <si>
-    <t>TTTTTCCCCTCCTAAGGAAGAGAG</t>
+    <t>GAAGGAGGAAGGAGAAGGAAAAGGAAAGGAGGGGAAAAA</t>
   </si>
   <si>
     <t>GAAGGAGGAAGGA</t>
@@ -343,7 +346,7 @@
     <t>AGGAGGGGAAAAA</t>
   </si>
   <si>
-    <t>GAAGGAGGAAGGAGAAGGAAAAGGAAAGGAGGGGAAAAA</t>
+    <t>TCCTTCCTCCTTCCCTCTTCCTTCTATCCTCTCTTCCTTTCCTTTTCCTTC</t>
   </si>
   <si>
     <t>TCCTTCCTCCTTC</t>
@@ -352,9 +355,6 @@
     <t>TTCCTTTTCCTTC</t>
   </si>
   <si>
-    <t>TCCTTCCTCCTTCCCTCTTCCTTCTATCCTCTCTTCCTTTCCTTTTCCTTC</t>
-  </si>
-  <si>
     <t>MiPTestGene_1244</t>
   </si>
   <si>
@@ -364,10 +364,13 @@
     <t>GAGAGAAGAGAAGGGGAGAGGAGAGGGAAGAAAAAGGGGA</t>
   </si>
   <si>
+    <t>TCCCCTTTTTCTTGAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>TCCCCTTTTTCTT</t>
   </si>
   <si>
-    <t>TCCCCTTTTTCTTGAGGAAGAGAG</t>
+    <t>GAGAGAAGAGAAGGGGAGAGGAGAGGAAGAAAAAGGGGA</t>
   </si>
   <si>
     <t>GAGAGAAGAGAAG</t>
@@ -379,7 +382,7 @@
     <t>AAGAAAAAGGGGA</t>
   </si>
   <si>
-    <t>GAGAGAAGAGAAGGGGAGAGGAGAGGAAGAAAAAGGGGA</t>
+    <t>CTTCTCTTCTCTCCCTCTTCCTTCTATCCTCTCTTCCTCCTCTCCTCTCCC</t>
   </si>
   <si>
     <t>CTTCTCTTCTCTC</t>
@@ -388,9 +391,6 @@
     <t>CCTCTCCTCTCCC</t>
   </si>
   <si>
-    <t>CTTCTCTTCTCTCCCTCTTCCTTCTATCCTCTCTTCCTCCTCTCCTCTCCC</t>
-  </si>
-  <si>
     <t>MiPTestGene_438</t>
   </si>
   <si>
@@ -400,10 +400,13 @@
     <t>GAGAAAGGAGAAGGAGGGGAGGAGAGGAAGAAGGGGGGAG</t>
   </si>
   <si>
+    <t>CTCCCCCCTTCTTGAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>CTCCCCCCTTCTT</t>
   </si>
   <si>
-    <t>CTCCCCCCTTCTTGAGGAAGAGAG</t>
+    <t>GAGAAAGGAGAAGGAGGGGAGGAGAGAAGAAGGGGGGAG</t>
   </si>
   <si>
     <t>GAGAAAGGAGAAG</t>
@@ -415,7 +418,7 @@
     <t>AAGAAGGGGGGAG</t>
   </si>
   <si>
-    <t>GAGAAAGGAGAAGGAGGGGAGGAGAGAAGAAGGGGGGAG</t>
+    <t>CTTCTCCTTTCTCCCTCTTCCTTCTATCCTCTCTTCCTCTCTCCTCCCCTC</t>
   </si>
   <si>
     <t>CTTCTCCTTTCTC</t>
@@ -424,9 +427,6 @@
     <t>CTCTCCTCCCCTC</t>
   </si>
   <si>
-    <t>CTTCTCCTTTCTCCCTCTTCCTTCTATCCTCTCTTCCTCTCTCCTCCCCTC</t>
-  </si>
-  <si>
     <t>MiPTestGene_1381</t>
   </si>
   <si>
@@ -436,10 +436,13 @@
     <t>GAAGGGAAGAAGGAAGAGAAGGGGAAGGAAAGGGAGGGGA</t>
   </si>
   <si>
+    <t>TCCCCTCCCTTTCGAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>TCCCCTCCCTTTC</t>
   </si>
   <si>
-    <t>TCCCCTCCCTTTCGAGGAAGAGAG</t>
+    <t>GAAGGGAAGAAGGAAGAGAAGGGGAAGAAAGGGAGGGGA</t>
   </si>
   <si>
     <t>GAAGGGAAGAAGG</t>
@@ -451,7 +454,7 @@
     <t>GAAAGGGAGGGGA</t>
   </si>
   <si>
-    <t>GAAGGGAAGAAGGAAGAGAAGGGGAAGAAAGGGAGGGGA</t>
+    <t>CCTTCTTCCCTTCCCTCTTCCTTCTATCCTCTCTTCCTTTCCCCTTCTCTT</t>
   </si>
   <si>
     <t>CCTTCTTCCCTTC</t>
@@ -460,9 +463,6 @@
     <t>TTCCCCTTCTCTT</t>
   </si>
   <si>
-    <t>CCTTCTTCCCTTCCCTCTTCCTTCTATCCTCTCTTCCTTTCCCCTTCTCTT</t>
-  </si>
-  <si>
     <t>MiPTestGene_571</t>
   </si>
   <si>
@@ -472,10 +472,13 @@
     <t>AGGAGGGAGGGAAGGAGGGAAAAGAGGAAAAGGAAAGGGG</t>
   </si>
   <si>
+    <t>CCCCTTTCCTTTTGAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>CCCCTTTCCTTTT</t>
   </si>
   <si>
-    <t>CCCCTTTCCTTTTGAGGAAGAGAG</t>
+    <t>AGGAGGGAGGGAAGGAGGGAAAAGAGAAAAGGAAAGGGG</t>
   </si>
   <si>
     <t>AGGAGGGAGGGAA</t>
@@ -487,7 +490,7 @@
     <t>AAAAGGAAAGGGG</t>
   </si>
   <si>
-    <t>AGGAGGGAGGGAAGGAGGGAAAAGAGAAAAGGAAAGGGG</t>
+    <t>TTCCCTCCCTCCTCCTCTTCCTTCTATCCTCTCTTCCTCTCTTTTCCCTCC</t>
   </si>
   <si>
     <t>TTCCCTCCCTCCT</t>
@@ -496,9 +499,6 @@
     <t>CTCTTTTCCCTCC</t>
   </si>
   <si>
-    <t>TTCCCTCCCTCCTCCTCTTCCTTCTATCCTCTCTTCCTCTCTTTTCCCTCC</t>
-  </si>
-  <si>
     <t>MiPTestGene_1473</t>
   </si>
   <si>
@@ -508,10 +508,13 @@
     <t>AAGAGAAGGAAGGAAGAAAAGGGAGGGAAAAAGAAAGGGG</t>
   </si>
   <si>
+    <t>CCCCTTTCTTTTTGAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>CCCCTTTCTTTTT</t>
   </si>
   <si>
-    <t>CCCCTTTCTTTTTGAGGAAGAGAG</t>
+    <t>AAGAGAAGGAAGGAAGAAAAGGGAGGAAAAAGAAAGGGG</t>
   </si>
   <si>
     <t>AAGAGAAGGAAGG</t>
@@ -523,7 +526,7 @@
     <t>AAAAAGAAAGGGG</t>
   </si>
   <si>
-    <t>AAGAGAAGGAAGGAAGAAAAGGGAGGAAAAAGAAAGGGG</t>
+    <t>CCTTCCTTCTCTTCCTCTTCCTTCTATCCTCTCTTCCTCCTCCCTTTTCTT</t>
   </si>
   <si>
     <t>CCTTCCTTCTCTT</t>
@@ -532,9 +535,6 @@
     <t>CCTCCCTTTTCTT</t>
   </si>
   <si>
-    <t>CCTTCCTTCTCTTCCTCTTCCTTCTATCCTCTCTTCCTCCTCCCTTTTCTT</t>
-  </si>
-  <si>
     <t>MiPTestGene_655</t>
   </si>
   <si>
@@ -544,10 +544,13 @@
     <t>GGAGAGAAGGGGAGGAAAGAAGGGAAGAAGAAAGGGGAAA</t>
   </si>
   <si>
+    <t>TTTCCCCTTTCTTGAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>TTTCCCCTTTCTT</t>
   </si>
   <si>
-    <t>TTTCCCCTTTCTTGAGGAAGAGAG</t>
+    <t>GGAGAGAAGGGGAGGAAAGAAGGGAAAAGAAAGGGGAAA</t>
   </si>
   <si>
     <t>GGAGAGAAGGGGA</t>
@@ -559,7 +562,7 @@
     <t>AAGAAAGGGGAAA</t>
   </si>
   <si>
-    <t>GGAGAGAAGGGGAGGAAAGAAGGGAAAAGAAAGGGGAAA</t>
+    <t>TCCCCTTCTCTCCCCTCTTCCTTCTATCCTCTCTTCCTTTCCCTTCTTTCC</t>
   </si>
   <si>
     <t>TCCCCTTCTCTCC</t>
@@ -568,9 +571,6 @@
     <t>TTCCCTTCTTTCC</t>
   </si>
   <si>
-    <t>TCCCCTTCTCTCCCCTCTTCCTTCTATCCTCTCTTCCTTTCCCTTCTTTCC</t>
-  </si>
-  <si>
     <t>MiPTestGene_1609</t>
   </si>
   <si>
@@ -580,10 +580,13 @@
     <t>GAAGAGAGGGAGGAAGGAAGAGGAAAGAGAAGAAAAGGGG</t>
   </si>
   <si>
+    <t>CCCCTTTTCTTCTGAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>CCCCTTTTCTTCT</t>
   </si>
   <si>
-    <t>CCCCTTTTCTTCTGAGGAAGAGAG</t>
+    <t>GAAGAGAGGGAGGAAGGAAGAGGAAAAGAAGAAAAGGGG</t>
   </si>
   <si>
     <t>GAAGAGAGGGAGG</t>
@@ -595,7 +598,7 @@
     <t>AGAAGAAAAGGGG</t>
   </si>
   <si>
-    <t>GAAGAGAGGGAGGAAGGAAGAGGAAAAGAAGAAAAGGGG</t>
+    <t>CCTCCCTCTCTTCCCTCTTCCTTCTATCCTCTCTTCCTTTTCCTCTTCCTT</t>
   </si>
   <si>
     <t>CCTCCCTCTCTTC</t>
@@ -604,9 +607,6 @@
     <t>TTTCCTCTTCCTT</t>
   </si>
   <si>
-    <t>CCTCCCTCTCTTCCCTCTTCCTTCTATCCTCTCTTCCTTTTCCTCTTCCTT</t>
-  </si>
-  <si>
     <t>MiPTestGene_1651</t>
   </si>
   <si>
@@ -616,10 +616,13 @@
     <t>GGGGGGAGAAGAGGGAGGAAAAGGGAAGGAGAAAAAAGGG</t>
   </si>
   <si>
+    <t>CCCTTTTTTCTCCAAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>CCCTTTTTTCTCC</t>
   </si>
   <si>
-    <t>CCCTTTTTTCTCCAAGGAAGAGAG</t>
+    <t>GGGGGGAGAAGAGGGAGGAAAAGGGAGGAGAAAAAAGGG</t>
   </si>
   <si>
     <t>GGGGGGAGAAGAG</t>
@@ -631,7 +634,7 @@
     <t>GGAGAAAAAAGGG</t>
   </si>
   <si>
-    <t>GGGGGGAGAAGAGGGAGGAAAAGGGAGGAGAAAAAAGGG</t>
+    <t>CTCTTCTCCCCCCCCTCTTCCTTCTATCCTCTCTTCCTTCCCTTTTCCTCC</t>
   </si>
   <si>
     <t>CTCTTCTCCCCCC</t>
@@ -640,9 +643,6 @@
     <t>TCCCTTTTCCTCC</t>
   </si>
   <si>
-    <t>CTCTTCTCCCCCCCCTCTTCCTTCTATCCTCTCTTCCTTCCCTTTTCCTCC</t>
-  </si>
-  <si>
     <t>MiPTestGene_830</t>
   </si>
   <si>
@@ -652,10 +652,13 @@
     <t>AGGGAGGGAGGAAAGGGAGGGAAGAGAGAAAGGGAGGGAG</t>
   </si>
   <si>
+    <t>CTCCCTCCCTTTCAAGGAAGAGAG</t>
+  </si>
+  <si>
     <t>CTCCCTCCCTTTC</t>
   </si>
   <si>
-    <t>CTCCCTCCCTTTCAAGGAAGAGAG</t>
+    <t>AGGGAGGGAGGAAAGGGAGGGAAGAGGAAAGGGAGGGAG</t>
   </si>
   <si>
     <t>AGGGAGGGAGGAA</t>
@@ -667,16 +670,13 @@
     <t>GAAAGGGAGGGAG</t>
   </si>
   <si>
-    <t>AGGGAGGGAGGAAAGGGAGGGAAGAGGAAAGGGAGGGAG</t>
+    <t>TTCCTCCCTCCCTCCTCTTCCTTCTATCCTCTCTTCCTCTCTTCCCTCCCT</t>
   </si>
   <si>
     <t>TTCCTCCCTCCCT</t>
   </si>
   <si>
     <t>CTCTTCCCTCCCT</t>
-  </si>
-  <si>
-    <t>TTCCTCCCTCCCTCCTCTTCCTTCTATCCTCTCTTCCTCTCTTCCCTCCCT</t>
   </si>
 </sst>
 </file>
@@ -751,7 +751,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1F8F4"/>
+        <fgColor rgb="FFF3F6FC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -763,7 +763,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF8EE"/>
+        <fgColor rgb="FFF1F8F4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -775,7 +775,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF7F3FC"/>
+        <fgColor rgb="FFFEF8EE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -787,7 +787,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3F6FC"/>
+        <fgColor rgb="FFF7F3FC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -832,7 +832,7 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -841,22 +841,22 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1162,10 +1162,15 @@
     <col min="1" max="2" width="27.7109375" customWidth="1"/>
     <col min="3" max="4" width="20.7109375" customWidth="1"/>
     <col min="5" max="5" width="27.7109375" customWidth="1"/>
-    <col min="6" max="6" width="48.7109375" customWidth="1"/>
-    <col min="7" max="7" width="20.7109375" customWidth="1"/>
-    <col min="8" max="21" width="48.7109375" customWidth="1"/>
-    <col min="22" max="30" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="48.7109375" customWidth="1"/>
+    <col min="8" max="9" width="20.7109375" customWidth="1"/>
+    <col min="10" max="13" width="48.7109375" customWidth="1"/>
+    <col min="14" max="15" width="20.7109375" customWidth="1"/>
+    <col min="16" max="19" width="48.7109375" customWidth="1"/>
+    <col min="20" max="22" width="20.7109375" customWidth="1"/>
+    <col min="23" max="28" width="48.7109375" customWidth="1"/>
+    <col min="29" max="30" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="26" customHeight="1">
@@ -1184,16 +1189,16 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="3" t="s">
@@ -1202,49 +1207,49 @@
       <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="T1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="U1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="V1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="4" t="s">
+      <c r="X1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Y1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="4" t="s">
+      <c r="Z1" s="5" t="s">
         <v>25</v>
       </c>
       <c r="AA1" s="5" t="s">
@@ -1253,10 +1258,10 @@
       <c r="AB1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AC1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AD1" s="5" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1276,80 +1281,80 @@
       <c r="E2" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="6">
+        <v>1</v>
+      </c>
+      <c r="G2" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="6">
-        <v>1</v>
-      </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I2" s="8">
+        <v>1</v>
+      </c>
+      <c r="J2" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="K2" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="L2" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="M2" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="N2" s="11">
+        <v>5.5</v>
+      </c>
+      <c r="O2" s="11">
+        <v>4</v>
+      </c>
+      <c r="P2" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="Q2" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="R2" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="O2" s="11" t="s">
+      <c r="S2" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="P2" s="12" t="s">
+      <c r="T2" s="14">
+        <v>39</v>
+      </c>
+      <c r="U2" s="14">
+        <v>38.51</v>
+      </c>
+      <c r="V2" s="14">
+        <v>40.16</v>
+      </c>
+      <c r="W2" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="Q2" s="12" t="s">
+      <c r="X2" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="R2" s="12" t="s">
+      <c r="Y2" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S2" s="12" t="s">
+      <c r="Z2" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T2" s="12" t="s">
+      <c r="AA2" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="U2" s="13" t="s">
+      <c r="AB2" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="V2" s="14">
-        <v>5.5</v>
-      </c>
-      <c r="W2" s="14">
-        <v>4</v>
-      </c>
-      <c r="X2" s="15">
-        <v>39</v>
-      </c>
-      <c r="Y2" s="15">
-        <v>38.51</v>
-      </c>
-      <c r="Z2" s="15">
-        <v>40.16</v>
-      </c>
-      <c r="AA2" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB2" s="16">
+      <c r="AC2" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD2" s="17">
         <v>0</v>
-      </c>
-      <c r="AC2" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD2" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:30">
@@ -1368,80 +1373,80 @@
       <c r="E3" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6">
+        <v>1</v>
+      </c>
+      <c r="G3" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G3" s="6">
-        <v>1</v>
-      </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I3" s="8">
+        <v>1</v>
+      </c>
+      <c r="J3" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J3" s="8" t="s">
+      <c r="K3" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L3" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="L3" s="10" t="s">
+      <c r="M3" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" s="11">
+        <v>4.6</v>
+      </c>
+      <c r="O3" s="11">
+        <v>4</v>
+      </c>
+      <c r="P3" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="M3" s="10" t="s">
+      <c r="Q3" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="N3" s="10" t="s">
+      <c r="R3" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="O3" s="11" t="s">
+      <c r="S3" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="P3" s="12" t="s">
+      <c r="T3" s="14">
+        <v>39.84</v>
+      </c>
+      <c r="U3" s="14">
+        <v>44.61</v>
+      </c>
+      <c r="V3" s="14">
+        <v>42.68</v>
+      </c>
+      <c r="W3" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="Q3" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R3" s="12" t="s">
+      <c r="X3" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y3" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S3" s="12" t="s">
+      <c r="Z3" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T3" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="U3" s="13" t="s">
+      <c r="AA3" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB3" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="V3" s="14">
-        <v>4.6</v>
-      </c>
-      <c r="W3" s="14">
-        <v>4</v>
-      </c>
-      <c r="X3" s="15">
-        <v>39.84</v>
-      </c>
-      <c r="Y3" s="15">
-        <v>44.61</v>
-      </c>
-      <c r="Z3" s="15">
-        <v>42.68</v>
-      </c>
-      <c r="AA3" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB3" s="16">
+      <c r="AC3" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD3" s="17">
         <v>0</v>
-      </c>
-      <c r="AC3" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD3" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:30">
@@ -1460,80 +1465,80 @@
       <c r="E4" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="6">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="G4" s="6">
-        <v>1</v>
-      </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I4" s="8">
+        <v>1</v>
+      </c>
+      <c r="J4" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="K4" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="J4" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="K4" s="9" t="s">
+      <c r="L4" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="L4" s="10" t="s">
+      <c r="M4" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N4" s="11">
+        <v>4</v>
+      </c>
+      <c r="O4" s="11">
+        <v>4</v>
+      </c>
+      <c r="P4" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="M4" s="10" t="s">
+      <c r="Q4" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="N4" s="10" t="s">
+      <c r="R4" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="O4" s="11" t="s">
+      <c r="S4" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="P4" s="12" t="s">
+      <c r="T4" s="14">
+        <v>39</v>
+      </c>
+      <c r="U4" s="14">
+        <v>41.19</v>
+      </c>
+      <c r="V4" s="14">
+        <v>44.61</v>
+      </c>
+      <c r="W4" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="Q4" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R4" s="12" t="s">
+      <c r="X4" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="Y4" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="Z4" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T4" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="U4" s="13" t="s">
+      <c r="AA4" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB4" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="V4" s="14">
-        <v>4</v>
-      </c>
-      <c r="W4" s="14">
-        <v>4</v>
-      </c>
-      <c r="X4" s="15">
-        <v>39</v>
-      </c>
-      <c r="Y4" s="15">
-        <v>41.19</v>
-      </c>
-      <c r="Z4" s="15">
-        <v>44.61</v>
-      </c>
-      <c r="AA4" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB4" s="16">
+      <c r="AC4" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD4" s="17">
         <v>0</v>
-      </c>
-      <c r="AC4" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD4" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:30">
@@ -1552,80 +1557,80 @@
       <c r="E5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="6">
+        <v>1</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="G5" s="6">
-        <v>1</v>
-      </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I5" s="8">
+        <v>1</v>
+      </c>
+      <c r="J5" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="I5" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J5" s="8" t="s">
+      <c r="K5" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="L5" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="K5" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="L5" s="10" t="s">
+      <c r="M5" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N5" s="11">
+        <v>6.1</v>
+      </c>
+      <c r="O5" s="11">
+        <v>4</v>
+      </c>
+      <c r="P5" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="M5" s="10" t="s">
+      <c r="Q5" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="N5" s="10" t="s">
+      <c r="R5" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="O5" s="11" t="s">
+      <c r="S5" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="P5" s="12" t="s">
+      <c r="T5" s="14">
+        <v>35.41</v>
+      </c>
+      <c r="U5" s="14">
+        <v>38.51</v>
+      </c>
+      <c r="V5" s="14">
+        <v>43.7</v>
+      </c>
+      <c r="W5" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="Q5" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R5" s="12" t="s">
+      <c r="X5" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y5" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S5" s="12" t="s">
+      <c r="Z5" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T5" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="U5" s="13" t="s">
+      <c r="AA5" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB5" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="V5" s="14">
-        <v>6.1</v>
-      </c>
-      <c r="W5" s="14">
-        <v>4</v>
-      </c>
-      <c r="X5" s="15">
-        <v>35.41</v>
-      </c>
-      <c r="Y5" s="15">
-        <v>38.51</v>
-      </c>
-      <c r="Z5" s="15">
-        <v>43.7</v>
-      </c>
-      <c r="AA5" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB5" s="16">
+      <c r="AC5" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD5" s="17">
         <v>0</v>
-      </c>
-      <c r="AC5" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD5" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:30">
@@ -1644,80 +1649,80 @@
       <c r="E6" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6">
+        <v>1</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="G6" s="6">
-        <v>1</v>
-      </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I6" s="8">
+        <v>1</v>
+      </c>
+      <c r="J6" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="I6" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="9" t="s">
+      <c r="K6" s="10" t="s">
         <v>92</v>
       </c>
       <c r="L6" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" s="11">
+        <v>4.6</v>
+      </c>
+      <c r="O6" s="11">
+        <v>4</v>
+      </c>
+      <c r="P6" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="M6" s="10" t="s">
+      <c r="Q6" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="N6" s="10" t="s">
+      <c r="R6" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="O6" s="11" t="s">
+      <c r="S6" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="P6" s="12" t="s">
+      <c r="T6" s="14">
+        <v>35.41</v>
+      </c>
+      <c r="U6" s="14">
+        <v>43.7</v>
+      </c>
+      <c r="V6" s="14">
+        <v>39.84</v>
+      </c>
+      <c r="W6" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="Q6" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R6" s="12" t="s">
+      <c r="X6" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y6" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S6" s="12" t="s">
+      <c r="Z6" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T6" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="U6" s="13" t="s">
+      <c r="AA6" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB6" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="V6" s="14">
-        <v>4.6</v>
-      </c>
-      <c r="W6" s="14">
-        <v>4</v>
-      </c>
-      <c r="X6" s="15">
-        <v>35.41</v>
-      </c>
-      <c r="Y6" s="15">
-        <v>43.7</v>
-      </c>
-      <c r="Z6" s="15">
-        <v>39.84</v>
-      </c>
-      <c r="AA6" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB6" s="16">
+      <c r="AC6" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD6" s="17">
         <v>0</v>
-      </c>
-      <c r="AC6" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD6" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:30">
@@ -1736,80 +1741,80 @@
       <c r="E7" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="6">
+        <v>1</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="G7" s="6">
-        <v>1</v>
-      </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I7" s="8">
+        <v>1</v>
+      </c>
+      <c r="J7" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="I7" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J7" s="8" t="s">
+      <c r="K7" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="L7" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="K7" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="L7" s="10" t="s">
+      <c r="M7" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N7" s="11">
+        <v>4.9</v>
+      </c>
+      <c r="O7" s="11">
+        <v>4</v>
+      </c>
+      <c r="P7" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="M7" s="10" t="s">
+      <c r="Q7" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="N7" s="10" t="s">
+      <c r="R7" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="O7" s="11" t="s">
+      <c r="S7" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="P7" s="12" t="s">
+      <c r="T7" s="14">
+        <v>40.16</v>
+      </c>
+      <c r="U7" s="14">
+        <v>35.54</v>
+      </c>
+      <c r="V7" s="14">
+        <v>39.84</v>
+      </c>
+      <c r="W7" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="Q7" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R7" s="12" t="s">
+      <c r="X7" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="Y7" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S7" s="12" t="s">
+      <c r="Z7" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T7" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="U7" s="13" t="s">
+      <c r="AA7" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB7" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="V7" s="14">
-        <v>4.9</v>
-      </c>
-      <c r="W7" s="14">
-        <v>4</v>
-      </c>
-      <c r="X7" s="15">
-        <v>40.16</v>
-      </c>
-      <c r="Y7" s="15">
-        <v>35.54</v>
-      </c>
-      <c r="Z7" s="15">
-        <v>39.84</v>
-      </c>
-      <c r="AA7" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB7" s="16">
+      <c r="AC7" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD7" s="17">
         <v>0</v>
-      </c>
-      <c r="AC7" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD7" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:30">
@@ -1828,80 +1833,80 @@
       <c r="E8" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="6">
+        <v>1</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="G8" s="6">
-        <v>1</v>
-      </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I8" s="8">
+        <v>1</v>
+      </c>
+      <c r="J8" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="I8" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="K8" s="9" t="s">
+      <c r="K8" s="10" t="s">
         <v>116</v>
       </c>
       <c r="L8" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="M8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N8" s="11">
+        <v>4.6</v>
+      </c>
+      <c r="O8" s="11">
+        <v>2</v>
+      </c>
+      <c r="P8" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="M8" s="10" t="s">
+      <c r="Q8" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="N8" s="10" t="s">
+      <c r="R8" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="O8" s="11" t="s">
+      <c r="S8" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="P8" s="12" t="s">
+      <c r="T8" s="14">
+        <v>35.09</v>
+      </c>
+      <c r="U8" s="14">
+        <v>43.91</v>
+      </c>
+      <c r="V8" s="14">
+        <v>37.04</v>
+      </c>
+      <c r="W8" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="Q8" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R8" s="12" t="s">
+      <c r="X8" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="Y8" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S8" s="12" t="s">
+      <c r="Z8" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T8" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="U8" s="13" t="s">
+      <c r="AA8" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB8" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="V8" s="14">
-        <v>4.6</v>
-      </c>
-      <c r="W8" s="14">
-        <v>2</v>
-      </c>
-      <c r="X8" s="15">
-        <v>35.09</v>
-      </c>
-      <c r="Y8" s="15">
-        <v>43.91</v>
-      </c>
-      <c r="Z8" s="15">
-        <v>37.04</v>
-      </c>
-      <c r="AA8" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB8" s="16">
+      <c r="AC8" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD8" s="17">
         <v>0</v>
-      </c>
-      <c r="AC8" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD8" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:30">
@@ -1920,80 +1925,80 @@
       <c r="E9" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="6">
+        <v>1</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="G9" s="6">
-        <v>1</v>
-      </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I9" s="8">
+        <v>1</v>
+      </c>
+      <c r="J9" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="K9" s="9" t="s">
+      <c r="K9" s="10" t="s">
         <v>128</v>
       </c>
       <c r="L9" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="M9" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N9" s="11">
+        <v>3.8</v>
+      </c>
+      <c r="O9" s="11">
+        <v>4</v>
+      </c>
+      <c r="P9" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="M9" s="10" t="s">
+      <c r="Q9" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="N9" s="10" t="s">
+      <c r="R9" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="O9" s="11" t="s">
+      <c r="S9" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="P9" s="12" t="s">
+      <c r="T9" s="14">
+        <v>35.87</v>
+      </c>
+      <c r="U9" s="14">
+        <v>43.91</v>
+      </c>
+      <c r="V9" s="14">
+        <v>43.7</v>
+      </c>
+      <c r="W9" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="Q9" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R9" s="12" t="s">
+      <c r="X9" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="Y9" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S9" s="12" t="s">
+      <c r="Z9" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T9" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="U9" s="13" t="s">
+      <c r="AA9" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB9" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="V9" s="14">
-        <v>3.8</v>
-      </c>
-      <c r="W9" s="14">
-        <v>4</v>
-      </c>
-      <c r="X9" s="15">
-        <v>35.87</v>
-      </c>
-      <c r="Y9" s="15">
-        <v>43.91</v>
-      </c>
-      <c r="Z9" s="15">
-        <v>43.7</v>
-      </c>
-      <c r="AA9" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB9" s="16">
+      <c r="AC9" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD9" s="17">
         <v>0</v>
-      </c>
-      <c r="AC9" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD9" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:30">
@@ -2012,80 +2017,80 @@
       <c r="E10" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="6">
+        <v>1</v>
+      </c>
+      <c r="G10" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="G10" s="6">
-        <v>1</v>
-      </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I10" s="8">
+        <v>1</v>
+      </c>
+      <c r="J10" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="I10" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="K10" s="9" t="s">
+      <c r="K10" s="10" t="s">
         <v>140</v>
       </c>
       <c r="L10" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="M10" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N10" s="11">
+        <v>5</v>
+      </c>
+      <c r="O10" s="11">
+        <v>3</v>
+      </c>
+      <c r="P10" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="M10" s="10" t="s">
+      <c r="Q10" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="N10" s="10" t="s">
+      <c r="R10" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="O10" s="11" t="s">
+      <c r="S10" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="P10" s="12" t="s">
+      <c r="T10" s="14">
+        <v>39.3</v>
+      </c>
+      <c r="U10" s="14">
+        <v>39</v>
+      </c>
+      <c r="V10" s="14">
+        <v>43.77</v>
+      </c>
+      <c r="W10" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="Q10" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R10" s="12" t="s">
+      <c r="X10" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y10" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S10" s="12" t="s">
+      <c r="Z10" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T10" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="U10" s="13" t="s">
+      <c r="AA10" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB10" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="V10" s="14">
-        <v>5</v>
-      </c>
-      <c r="W10" s="14">
-        <v>3</v>
-      </c>
-      <c r="X10" s="15">
-        <v>39.3</v>
-      </c>
-      <c r="Y10" s="15">
-        <v>39</v>
-      </c>
-      <c r="Z10" s="15">
-        <v>43.77</v>
-      </c>
-      <c r="AA10" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB10" s="16">
+      <c r="AC10" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD10" s="17">
         <v>0</v>
-      </c>
-      <c r="AC10" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD10" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:30">
@@ -2104,80 +2109,80 @@
       <c r="E11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="6">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="G11" s="6">
-        <v>1</v>
-      </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I11" s="8">
+        <v>1</v>
+      </c>
+      <c r="J11" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="I11" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="10" t="s">
         <v>152</v>
       </c>
       <c r="L11" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="M11" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N11" s="11">
+        <v>4.4</v>
+      </c>
+      <c r="O11" s="11">
+        <v>4</v>
+      </c>
+      <c r="P11" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="M11" s="10" t="s">
+      <c r="Q11" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="N11" s="10" t="s">
+      <c r="R11" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="O11" s="11" t="s">
+      <c r="S11" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="P11" s="12" t="s">
+      <c r="T11" s="14">
+        <v>44.7</v>
+      </c>
+      <c r="U11" s="14">
+        <v>39.3</v>
+      </c>
+      <c r="V11" s="14">
+        <v>38.97</v>
+      </c>
+      <c r="W11" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="Q11" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R11" s="12" t="s">
+      <c r="X11" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="Y11" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S11" s="12" t="s">
+      <c r="Z11" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T11" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="U11" s="13" t="s">
+      <c r="AA11" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB11" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="V11" s="14">
-        <v>4.4</v>
-      </c>
-      <c r="W11" s="14">
-        <v>4</v>
-      </c>
-      <c r="X11" s="15">
-        <v>44.7</v>
-      </c>
-      <c r="Y11" s="15">
-        <v>39.3</v>
-      </c>
-      <c r="Z11" s="15">
-        <v>38.97</v>
-      </c>
-      <c r="AA11" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB11" s="16">
+      <c r="AC11" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD11" s="17">
         <v>0</v>
-      </c>
-      <c r="AC11" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD11" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:30">
@@ -2196,80 +2201,80 @@
       <c r="E12" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="6">
+        <v>1</v>
+      </c>
+      <c r="G12" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="G12" s="6">
-        <v>1</v>
-      </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I12" s="8">
+        <v>1</v>
+      </c>
+      <c r="J12" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="I12" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="K12" s="9" t="s">
+      <c r="K12" s="10" t="s">
         <v>164</v>
       </c>
       <c r="L12" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N12" s="11">
+        <v>5.6</v>
+      </c>
+      <c r="O12" s="11">
+        <v>2</v>
+      </c>
+      <c r="P12" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="M12" s="10" t="s">
+      <c r="Q12" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="N12" s="10" t="s">
+      <c r="R12" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="O12" s="11" t="s">
+      <c r="S12" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="P12" s="12" t="s">
+      <c r="T12" s="14">
+        <v>37.34</v>
+      </c>
+      <c r="U12" s="14">
+        <v>38.15</v>
+      </c>
+      <c r="V12" s="14">
+        <v>36.24</v>
+      </c>
+      <c r="W12" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="Q12" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R12" s="12" t="s">
+      <c r="X12" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="Y12" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S12" s="12" t="s">
+      <c r="Z12" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T12" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="U12" s="13" t="s">
+      <c r="AA12" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB12" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="V12" s="14">
-        <v>5.6</v>
-      </c>
-      <c r="W12" s="14">
-        <v>2</v>
-      </c>
-      <c r="X12" s="15">
-        <v>37.34</v>
-      </c>
-      <c r="Y12" s="15">
-        <v>38.15</v>
-      </c>
-      <c r="Z12" s="15">
-        <v>36.24</v>
-      </c>
-      <c r="AA12" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB12" s="16">
+      <c r="AC12" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD12" s="17">
         <v>0</v>
-      </c>
-      <c r="AC12" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD12" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:30">
@@ -2288,80 +2293,80 @@
       <c r="E13" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="6">
+        <v>1</v>
+      </c>
+      <c r="G13" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="G13" s="6">
-        <v>1</v>
-      </c>
-      <c r="H13" s="8" t="s">
+      <c r="H13" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I13" s="8">
+        <v>1</v>
+      </c>
+      <c r="J13" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="I13" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="K13" s="9" t="s">
+      <c r="K13" s="10" t="s">
         <v>176</v>
       </c>
       <c r="L13" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N13" s="11">
+        <v>5.6</v>
+      </c>
+      <c r="O13" s="11">
+        <v>4</v>
+      </c>
+      <c r="P13" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="M13" s="10" t="s">
+      <c r="Q13" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="N13" s="10" t="s">
+      <c r="R13" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="O13" s="11" t="s">
+      <c r="S13" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="P13" s="12" t="s">
+      <c r="T13" s="14">
+        <v>42.93</v>
+      </c>
+      <c r="U13" s="14">
+        <v>38.24</v>
+      </c>
+      <c r="V13" s="14">
+        <v>37.04</v>
+      </c>
+      <c r="W13" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="Q13" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R13" s="12" t="s">
+      <c r="X13" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="Y13" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S13" s="12" t="s">
+      <c r="Z13" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T13" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="U13" s="13" t="s">
+      <c r="AA13" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB13" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="V13" s="14">
-        <v>5.6</v>
-      </c>
-      <c r="W13" s="14">
-        <v>4</v>
-      </c>
-      <c r="X13" s="15">
-        <v>42.93</v>
-      </c>
-      <c r="Y13" s="15">
-        <v>38.24</v>
-      </c>
-      <c r="Z13" s="15">
-        <v>37.04</v>
-      </c>
-      <c r="AA13" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB13" s="16">
+      <c r="AC13" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD13" s="17">
         <v>0</v>
-      </c>
-      <c r="AC13" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD13" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:30">
@@ -2380,80 +2385,80 @@
       <c r="E14" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="6">
+        <v>1</v>
+      </c>
+      <c r="G14" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="G14" s="6">
-        <v>1</v>
-      </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I14" s="8">
+        <v>1</v>
+      </c>
+      <c r="J14" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="I14" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J14" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="K14" s="9" t="s">
+      <c r="K14" s="10" t="s">
         <v>188</v>
       </c>
       <c r="L14" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="M14" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N14" s="11">
+        <v>5.6</v>
+      </c>
+      <c r="O14" s="11">
+        <v>4</v>
+      </c>
+      <c r="P14" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="M14" s="10" t="s">
+      <c r="Q14" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="N14" s="10" t="s">
+      <c r="R14" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="O14" s="11" t="s">
+      <c r="S14" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="P14" s="12" t="s">
+      <c r="T14" s="14">
+        <v>41.19</v>
+      </c>
+      <c r="U14" s="14">
+        <v>36.22</v>
+      </c>
+      <c r="V14" s="14">
+        <v>38.15</v>
+      </c>
+      <c r="W14" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="Q14" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R14" s="12" t="s">
+      <c r="X14" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="Y14" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S14" s="12" t="s">
+      <c r="Z14" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T14" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="U14" s="13" t="s">
+      <c r="AA14" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB14" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="V14" s="14">
-        <v>5.6</v>
-      </c>
-      <c r="W14" s="14">
-        <v>4</v>
-      </c>
-      <c r="X14" s="15">
-        <v>41.19</v>
-      </c>
-      <c r="Y14" s="15">
-        <v>36.22</v>
-      </c>
-      <c r="Z14" s="15">
-        <v>38.15</v>
-      </c>
-      <c r="AA14" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB14" s="16">
+      <c r="AC14" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD14" s="17">
         <v>0</v>
-      </c>
-      <c r="AC14" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD14" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:30">
@@ -2472,80 +2477,80 @@
       <c r="E15" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="6">
+        <v>1</v>
+      </c>
+      <c r="G15" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="G15" s="6">
-        <v>1</v>
-      </c>
-      <c r="H15" s="8" t="s">
+      <c r="H15" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I15" s="8">
+        <v>1</v>
+      </c>
+      <c r="J15" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="I15" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J15" s="8" t="s">
+      <c r="K15" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="L15" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="K15" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="L15" s="10" t="s">
+      <c r="M15" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N15" s="11">
+        <v>6.2</v>
+      </c>
+      <c r="O15" s="11">
+        <v>4</v>
+      </c>
+      <c r="P15" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="M15" s="10" t="s">
+      <c r="Q15" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="N15" s="10" t="s">
+      <c r="R15" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="O15" s="11" t="s">
+      <c r="S15" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="P15" s="12" t="s">
+      <c r="T15" s="14">
+        <v>44.74</v>
+      </c>
+      <c r="U15" s="14">
+        <v>40.98</v>
+      </c>
+      <c r="V15" s="14">
+        <v>37.43</v>
+      </c>
+      <c r="W15" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="Q15" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R15" s="12" t="s">
+      <c r="X15" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="Y15" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S15" s="12" t="s">
+      <c r="Z15" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T15" s="12" t="s">
-        <v>206</v>
-      </c>
-      <c r="U15" s="13" t="s">
+      <c r="AA15" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB15" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="V15" s="14">
-        <v>6.2</v>
-      </c>
-      <c r="W15" s="14">
-        <v>4</v>
-      </c>
-      <c r="X15" s="15">
-        <v>44.74</v>
-      </c>
-      <c r="Y15" s="15">
-        <v>40.98</v>
-      </c>
-      <c r="Z15" s="15">
-        <v>37.43</v>
-      </c>
-      <c r="AA15" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB15" s="16">
+      <c r="AC15" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD15" s="17">
         <v>0</v>
-      </c>
-      <c r="AC15" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD15" s="17">
-        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:30">
@@ -2564,80 +2569,80 @@
       <c r="E16" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="6">
+        <v>1</v>
+      </c>
+      <c r="G16" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="G16" s="6">
-        <v>1</v>
-      </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="8">
+        <v>-0</v>
+      </c>
+      <c r="I16" s="8">
+        <v>1</v>
+      </c>
+      <c r="J16" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="I16" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J16" s="8" t="s">
+      <c r="K16" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="L16" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="K16" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="L16" s="10" t="s">
+      <c r="M16" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N16" s="11">
+        <v>5.1</v>
+      </c>
+      <c r="O16" s="11">
+        <v>2</v>
+      </c>
+      <c r="P16" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="M16" s="10" t="s">
+      <c r="Q16" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="N16" s="10" t="s">
+      <c r="R16" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="O16" s="11" t="s">
+      <c r="S16" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="P16" s="12" t="s">
+      <c r="T16" s="14">
+        <v>44.7</v>
+      </c>
+      <c r="U16" s="14">
+        <v>42.86</v>
+      </c>
+      <c r="V16" s="14">
+        <v>42</v>
+      </c>
+      <c r="W16" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="Q16" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="R16" s="12" t="s">
+      <c r="X16" s="16" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y16" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S16" s="12" t="s">
+      <c r="Z16" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="T16" s="12" t="s">
-        <v>218</v>
-      </c>
-      <c r="U16" s="13" t="s">
+      <c r="AA16" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB16" s="16" t="s">
         <v>219</v>
       </c>
-      <c r="V16" s="14">
-        <v>5.1</v>
-      </c>
-      <c r="W16" s="14">
-        <v>2</v>
-      </c>
-      <c r="X16" s="15">
-        <v>44.7</v>
-      </c>
-      <c r="Y16" s="15">
-        <v>42.86</v>
-      </c>
-      <c r="Z16" s="15">
-        <v>42</v>
-      </c>
-      <c r="AA16" s="16">
-        <v>-0</v>
-      </c>
-      <c r="AB16" s="16">
+      <c r="AC16" s="17">
+        <v>-0</v>
+      </c>
+      <c r="AD16" s="17">
         <v>0</v>
-      </c>
-      <c r="AC16" s="17">
-        <v>-0</v>
-      </c>
-      <c r="AD16" s="17">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>